<commit_message>
Introduce a staged upload flow with AI-powered validation
Introduce a new staged upload process that allows files to be validated by an AI gatekeeper before being committed. This includes updates to parsing logic, API endpoints, database schema, and UI components.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 973c8810-ef52-4871-90e4-4a3959132a83
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 72cdf06c-a4d0-461f-af70-e0531e1d8476
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/168f086a-b8f0-4651-b359-6b33f4c435ed/973c8810-ef52-4871-90e4-4a3959132a83/4J3y22P
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/DATA_STRUCTURE.xlsx
+++ b/docs/DATA_STRUCTURE.xlsx
@@ -9,10 +9,11 @@
     <sheet name="Table - imports" sheetId="4" r:id="rId4"/>
     <sheet name="Table - record_pool" sheetId="5" r:id="rId5"/>
     <sheet name="Table - import_rows" sheetId="6" r:id="rId6"/>
-    <sheet name="ParseSummary" sheetId="7" r:id="rId7"/>
-    <sheet name="ChangeSummary" sheetId="8" r:id="rId8"/>
-    <sheet name="Computed Fields" sheetId="9" r:id="rId9"/>
-    <sheet name="API Endpoints" sheetId="10" r:id="rId10"/>
+    <sheet name="Table - upload_staging" sheetId="7" r:id="rId7"/>
+    <sheet name="ParseSummary" sheetId="8" r:id="rId8"/>
+    <sheet name="ChangeSummary" sheetId="9" r:id="rId9"/>
+    <sheet name="Computed Fields" sheetId="10" r:id="rId10"/>
+    <sheet name="API Endpoints" sheetId="11" r:id="rId11"/>
   </sheets>
 </workbook>
 </file>
@@ -435,7 +436,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Header is on row 3. Fill data from row 4 onward. Keep these column names exactly.</v>
+        <v>Header row is auto-detected (the row containing 'Project Code'); data starts on the next row. Keep these column names exactly.</v>
       </c>
     </row>
     <row r="3">
@@ -671,7 +672,83 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C6"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="56.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Recomputed on every read (not stored)</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Field</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Type</v>
+      </c>
+      <c r="C2" t="str">
+        <v>How it is computed</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>ageingDays</v>
+      </c>
+      <c r="B3" t="str">
+        <v>integer/null</v>
+      </c>
+      <c r="C3" t="str">
+        <v>today - assignDate in whole UTC days; null if no date</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>ageing color</v>
+      </c>
+      <c r="B4" t="str">
+        <v>n/a</v>
+      </c>
+      <c r="C4" t="str">
+        <v>green &lt;=30, amber 31-60, red &gt;60, neutral when no date</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>routeSteps</v>
+      </c>
+      <c r="B5" t="str">
+        <v>string[]</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Operation string split on commas (trimmed)</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>currentStepIndex</v>
+      </c>
+      <c r="B6" t="str">
+        <v>integer/null</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Index of activity within routeSteps, else null</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C18"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="44.83203125" customWidth="1"/>
@@ -719,122 +796,166 @@
         <v>multipart: file (req), label, reportDate</v>
       </c>
       <c r="C4" t="str">
-        <v>Created import + change set</v>
+        <v>Created import + change set (direct, no gate)</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>DELETE /imports</v>
+        <v>POST /imports/stage</v>
       </c>
       <c r="B5" t="str">
-        <v>none</v>
+        <v>multipart: file (req), label, reportDate</v>
       </c>
       <c r="C5" t="str">
-        <v>{ importsDeleted, poolRowsDeleted } — full reset</v>
+        <v>{ stagingId, sourceFilename, structural } — holds the file; nothing committed</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>GET /imports/{id}</v>
+        <v>POST /imports/validate</v>
       </c>
       <c r="B6" t="str">
-        <v>path id</v>
+        <v>json { stagingId }</v>
       </c>
       <c r="C6" t="str">
-        <v>One import with summaries</v>
+        <v>Gatekeeper verdict (ok/reject) + descriptive-only sanitize suggestions (advisory)</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>DELETE /imports/{id}</v>
+        <v>POST /imports/commit</v>
       </c>
       <c r="B7" t="str">
-        <v>path id</v>
+        <v>json { stagingId, acceptedSuggestions? }</v>
       </c>
       <c r="C7" t="str">
-        <v>204; deletes the import only (pool stays)</v>
+        <v>Applies accepted (field,from)-&gt;to cleanups, merges, returns created import + change set</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>GET /imports/{id}/records</v>
+        <v>DELETE /imports/stage/{id}</v>
       </c>
       <c r="B8" t="str">
         <v>path id</v>
       </c>
       <c r="C8" t="str">
-        <v>Records, copy-expanded, with live ageing/route</v>
+        <v>204; discards a staged upload without committing</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>GET /imports/{id}/changes</v>
+        <v>DELETE /imports</v>
       </c>
       <c r="B9" t="str">
-        <v>path id</v>
+        <v>none</v>
       </c>
       <c r="C9" t="str">
-        <v>Change set vs previous import</v>
+        <v>{ importsDeleted, poolRowsDeleted } — full reset</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>GET /imports/compare</v>
+        <v>GET /imports/{id}</v>
       </c>
       <c r="B10" t="str">
-        <v>query from (req), to (req)</v>
+        <v>path id</v>
       </c>
       <c r="C10" t="str">
-        <v>Change set between any two imports</v>
+        <v>One import with summaries</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>GET /ai/status</v>
+        <v>DELETE /imports/{id}</v>
       </c>
       <c r="B11" t="str">
-        <v>none</v>
+        <v>path id</v>
       </c>
       <c r="C11" t="str">
-        <v>{ available }</v>
+        <v>204; deletes the import only (pool stays)</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>POST /ai/sanitize</v>
+        <v>GET /imports/{id}/records</v>
       </c>
       <c r="B12" t="str">
-        <v>json { importId }</v>
+        <v>path id</v>
       </c>
       <c r="C12" t="str">
-        <v>Suggested descriptive-field cleanups (advisory)</v>
+        <v>Records, copy-expanded, with live ageing/route</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>POST /ai/review</v>
+        <v>GET /imports/{id}/changes</v>
       </c>
       <c r="B13" t="str">
-        <v>json { importId, compareTo?, deep? }</v>
+        <v>path id</v>
       </c>
       <c r="C13" t="str">
-        <v>Consistency audit (advisory, read-only)</v>
+        <v>Change set vs previous import</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
+        <v>GET /imports/compare</v>
+      </c>
+      <c r="B14" t="str">
+        <v>query from (req), to (req)</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Change set between any two imports</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>GET /ai/status</v>
+      </c>
+      <c r="B15" t="str">
+        <v>none</v>
+      </c>
+      <c r="C15" t="str">
+        <v>{ available }</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>POST /ai/sanitize</v>
+      </c>
+      <c r="B16" t="str">
+        <v>json { importId }</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Suggested descriptive-field cleanups (advisory)</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>POST /ai/review</v>
+      </c>
+      <c r="B17" t="str">
+        <v>json { importId, compareTo?, deep? }</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Consistency audit (advisory, read-only)</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
         <v>POST /ai/report</v>
       </c>
-      <c r="B14" t="str">
+      <c r="B18" t="str">
         <v>json { importId, compareTo?, filters? }</v>
       </c>
-      <c r="C14" t="str">
+      <c r="C18" t="str">
         <v>Turnaround analytical report (advisory)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C18"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1375,7 +1496,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C29"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -1417,7 +1538,7 @@
         <v>text unique</v>
       </c>
       <c r="C4" t="str">
-        <v>SHA-256 of all 18 normalized fields; identical rows share it</v>
+        <v>SHA-256 of the original 18 source fields; identical rows share it (derived mark fields excluded)</v>
       </c>
     </row>
     <row r="5">
@@ -1439,7 +1560,7 @@
         <v>text</v>
       </c>
       <c r="C6" t="str">
-        <v>Derived from Alias</v>
+        <v>= alias_corrected</v>
       </c>
     </row>
     <row r="7">
@@ -1450,7 +1571,7 @@
         <v>text</v>
       </c>
       <c r="C7" t="str">
-        <v>Mark No. with '&lt;job&gt; &lt;alias&gt;-' prefix stripped</v>
+        <v>= m_no</v>
       </c>
     </row>
     <row r="8">
@@ -1461,199 +1582,243 @@
         <v>text</v>
       </c>
       <c r="C8" t="str">
-        <v>job\structure\markTail (human-facing identity)</v>
+        <v>= mark_number (human-facing + change-log identity)</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>order_nature</v>
+        <v>m_no</v>
       </c>
       <c r="B9" t="str">
-        <v>text/null</v>
+        <v>text</v>
       </c>
       <c r="C9" t="str">
-        <v>Order Nature</v>
+        <v>Parsed bare mark tail (e.g. M101); notNull default ''</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>contractor</v>
+        <v>project_suffix</v>
       </c>
       <c r="B10" t="str">
-        <v>text/null</v>
+        <v>text</v>
       </c>
       <c r="C10" t="str">
-        <v>Contractor</v>
+        <v>Project segment of a backslash mark, else ''; notNull default ''</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>job_card_no</v>
+        <v>alias_corrected</v>
       </c>
       <c r="B11" t="str">
-        <v>text/null</v>
+        <v>text</v>
       </c>
       <c r="C11" t="str">
-        <v>Job Card No.</v>
+        <v>Structure/alias resolved from the mark (falls back to Alias); notNull default ''</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>tower_type</v>
+        <v>mark_number</v>
       </c>
       <c r="B12" t="str">
-        <v>text/null</v>
+        <v>text</v>
       </c>
       <c r="C12" t="str">
-        <v>Tower Type</v>
+        <v>job\alias_corrected\m_no (canonical backslash identity); notNull default ''</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>tower_sub_type</v>
+        <v>order_nature</v>
       </c>
       <c r="B13" t="str">
         <v>text/null</v>
       </c>
       <c r="C13" t="str">
-        <v>Tower Sub Type</v>
+        <v>Order Nature</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>alias</v>
+        <v>contractor</v>
       </c>
       <c r="B14" t="str">
         <v>text/null</v>
       </c>
       <c r="C14" t="str">
-        <v>Alias</v>
+        <v>Contractor</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>mark_no</v>
+        <v>job_card_no</v>
       </c>
       <c r="B15" t="str">
-        <v>text</v>
+        <v>text/null</v>
       </c>
       <c r="C15" t="str">
-        <v>Mark No. (raw)</v>
+        <v>Job Card No.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>section</v>
+        <v>tower_type</v>
       </c>
       <c r="B16" t="str">
         <v>text/null</v>
       </c>
       <c r="C16" t="str">
-        <v>Section</v>
+        <v>Tower Type</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>length</v>
+        <v>tower_sub_type</v>
       </c>
       <c r="B17" t="str">
-        <v>number/null</v>
+        <v>text/null</v>
       </c>
       <c r="C17" t="str">
-        <v>Length</v>
+        <v>Tower Sub Type</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>width</v>
+        <v>alias</v>
       </c>
       <c r="B18" t="str">
-        <v>number/null</v>
+        <v>text/null</v>
       </c>
       <c r="C18" t="str">
-        <v>Width</v>
+        <v>Alias</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>wt_pcs</v>
+        <v>mark_no</v>
       </c>
       <c r="B19" t="str">
-        <v>number/null</v>
+        <v>text</v>
       </c>
       <c r="C19" t="str">
-        <v>Wt/Pcs</v>
+        <v>Mark No. (raw)</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>balance_qty</v>
+        <v>section</v>
       </c>
       <c r="B20" t="str">
-        <v>number</v>
+        <v>text/null</v>
       </c>
       <c r="C20" t="str">
-        <v>Balance Qty. (defaults 0)</v>
+        <v>Section</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>balance_wt</v>
+        <v>length</v>
       </c>
       <c r="B21" t="str">
-        <v>number</v>
+        <v>number/null</v>
       </c>
       <c r="C21" t="str">
-        <v>Balance Wt. (defaults 0)</v>
+        <v>Length</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>assign_date</v>
+        <v>width</v>
       </c>
       <c r="B22" t="str">
-        <v>date/null</v>
+        <v>number/null</v>
       </c>
       <c r="C22" t="str">
-        <v>Assign Date, normalized YYYY-MM-DD</v>
+        <v>Width</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>activity</v>
+        <v>wt_pcs</v>
       </c>
       <c r="B23" t="str">
-        <v>text/null</v>
+        <v>number/null</v>
       </c>
       <c r="C23" t="str">
-        <v>Activity</v>
+        <v>Wt/Pcs</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>operation</v>
+        <v>balance_qty</v>
       </c>
       <c r="B24" t="str">
-        <v>text/null</v>
+        <v>number</v>
       </c>
       <c r="C24" t="str">
-        <v>Operation</v>
+        <v>Balance Qty. (defaults 0)</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
+        <v>balance_wt</v>
+      </c>
+      <c r="B25" t="str">
+        <v>number</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Balance Wt. (defaults 0)</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>assign_date</v>
+      </c>
+      <c r="B26" t="str">
+        <v>date/null</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Assign Date, normalized YYYY-MM-DD</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>activity</v>
+      </c>
+      <c r="B27" t="str">
+        <v>text/null</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Activity</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>operation</v>
+      </c>
+      <c r="B28" t="str">
+        <v>text/null</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Operation</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
         <v>ref_job_card_no</v>
       </c>
-      <c r="B25" t="str">
+      <c r="B29" t="str">
         <v>text/null</v>
       </c>
-      <c r="C25" t="str">
+      <c r="C29" t="str">
         <v>Ref. Job Card No.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C29"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1725,6 +1890,104 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C8"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="56.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Temporary holding for the gatekeeper flow; nothing is committed until the user accepts. Removed on commit or discard.</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Column</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Type</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Description</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>id</v>
+      </c>
+      <c r="B3" t="str">
+        <v>text (uuid) PK</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Staging id returned by POST /imports/stage</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>source_filename</v>
+      </c>
+      <c r="B4" t="str">
+        <v>text</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Original file name</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>label</v>
+      </c>
+      <c r="B5" t="str">
+        <v>text/null</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Friendly name (optional)</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>report_date</v>
+      </c>
+      <c r="B6" t="str">
+        <v>date/null</v>
+      </c>
+      <c r="C6" t="str">
+        <v>'As of' date (optional)</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>file_data</v>
+      </c>
+      <c r="B7" t="str">
+        <v>bytea</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Raw uploaded .xlsx bytes</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>created_at</v>
+      </c>
+      <c r="B8" t="str">
+        <v>timestamp</v>
+      </c>
+      <c r="C8" t="str">
+        <v>When it was staged</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C9"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
@@ -1832,7 +2095,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C12"/>
   <cols>
@@ -1972,80 +2235,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
-  <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="56.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Recomputed on every read (not stored)</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Field</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Type</v>
-      </c>
-      <c r="C2" t="str">
-        <v>How it is computed</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>ageingDays</v>
-      </c>
-      <c r="B3" t="str">
-        <v>integer/null</v>
-      </c>
-      <c r="C3" t="str">
-        <v>today - assignDate in whole UTC days; null if no date</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>ageing color</v>
-      </c>
-      <c r="B4" t="str">
-        <v>n/a</v>
-      </c>
-      <c r="C4" t="str">
-        <v>green &lt;=30, amber 31-60, red &gt;60, neutral when no date</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>routeSteps</v>
-      </c>
-      <c r="B5" t="str">
-        <v>string[]</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Operation string split on commas (trimmed)</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>currentStepIndex</v>
-      </c>
-      <c r="B6" t="str">
-        <v>integer/null</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Index of activity within routeSteps, else null</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>